<commit_message>
Updated resistors to correct 0805 case
</commit_message>
<xml_diff>
--- a/B+ Delay/bom_mouser_2025_06.xlsx
+++ b/B+ Delay/bom_mouser_2025_06.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2220866c56961e57/Documents/git_repos/B^M Delay/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2220866c56961e57/Documents/GitHub/B-HeaterDelay/B^M Delay/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="8_{83DCB168-53FD-4C0F-B771-7A2A33DAB321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E338634-8E16-466B-BB6D-02D907EE955B}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="8_{83DCB168-53FD-4C0F-B771-7A2A33DAB321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5EEBA68-2D23-4236-A7F8-F899903BDFA6}"/>
   <bookViews>
-    <workbookView xWindow="75" yWindow="1365" windowWidth="11145" windowHeight="11295" xr2:uid="{A484D203-BB89-4406-8269-6F9488CE3ED6}"/>
+    <workbookView xWindow="12060" yWindow="3825" windowWidth="21600" windowHeight="11190" xr2:uid="{A484D203-BB89-4406-8269-6F9488CE3ED6}"/>
   </bookViews>
   <sheets>
-    <sheet name="bom_mouser_2025_06" sheetId="1" r:id="rId1"/>
+    <sheet name="bom_mouser_2025_12" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="76">
   <si>
     <t>Designator</t>
   </si>
@@ -28,9 +28,6 @@
     <t>Footprint</t>
   </si>
   <si>
-    <t>Quantity</t>
-  </si>
-  <si>
     <t>Value</t>
   </si>
   <si>
@@ -172,9 +169,6 @@
     <t>CPC1779</t>
   </si>
   <si>
-    <t>Mouser</t>
-  </si>
-  <si>
     <t>845-29.002</t>
   </si>
   <si>
@@ -199,18 +193,12 @@
     <t>621-DF01ST</t>
   </si>
   <si>
-    <t>L7805ABD2T-TR</t>
-  </si>
-  <si>
     <t>849-CPC1779J</t>
   </si>
   <si>
     <t>595-NE556DR</t>
   </si>
   <si>
-    <t>MMBT3904637-MMBT3904</t>
-  </si>
-  <si>
     <t>637-MMBT3906</t>
   </si>
   <si>
@@ -226,22 +214,40 @@
     <t>71-CRCW080510K0JNEB</t>
   </si>
   <si>
-    <t>71-CRCW0402470KFKED</t>
-  </si>
-  <si>
-    <t>71-CRCW0402-4.12K-E3</t>
-  </si>
-  <si>
-    <t>71-CRCW0402200KFKEE</t>
-  </si>
-  <si>
-    <t>71-CRCW0402-60.4-E3</t>
-  </si>
-  <si>
     <t>667-EEE-FK1A102GP</t>
   </si>
   <si>
     <t>667-EEE-FK1K470P</t>
+  </si>
+  <si>
+    <t>652-CR0805FX-4121ELF</t>
+  </si>
+  <si>
+    <t>652-CR0805JW-474ELF</t>
+  </si>
+  <si>
+    <t>652-CR0805FX-68R0ELF</t>
+  </si>
+  <si>
+    <t>652-CR0805FX-2003ELF</t>
+  </si>
+  <si>
+    <t>637-MMBT3904</t>
+  </si>
+  <si>
+    <t>MMBT3904</t>
+  </si>
+  <si>
+    <t>621-AS7805ADTR-G1</t>
+  </si>
+  <si>
+    <t>Mouser Part Number</t>
+  </si>
+  <si>
+    <t>Quantity used</t>
+  </si>
+  <si>
+    <t>Quantity Order</t>
   </si>
 </sst>
 </file>
@@ -597,7 +603,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -713,9 +719,22 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FFD9D9D9"/>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right/>
       <top/>
       <bottom style="medium">
@@ -769,21 +788,20 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="42"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1" indent="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="42" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -841,10 +859,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1164,388 +1178,419 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4664FE7-DAA6-4A8C-B11D-C1FF94B408C0}">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="15.5703125" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="5" max="5" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.140625" customWidth="1"/>
+    <col min="6" max="6" width="22.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="B2" s="3">
+        <v>805</v>
+      </c>
+      <c r="C2" s="3">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="3">
+        <v>805</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="3">
+        <v>1210</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="3">
+        <v>805</v>
+      </c>
+      <c r="C7" s="3">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="3">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2">
+      <c r="B9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="3">
+        <v>2</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="3">
+        <v>2</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="3">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="3">
+        <v>1</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="3">
         <v>805</v>
       </c>
-      <c r="C2">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="C13" s="3">
+        <v>1</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="3">
+        <v>805</v>
+      </c>
+      <c r="C14" s="3">
+        <v>1</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="3">
+        <v>805</v>
+      </c>
+      <c r="C15" s="3">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="3">
+        <v>805</v>
+      </c>
+      <c r="C16" s="3">
+        <v>3</v>
+      </c>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="3">
+        <v>805</v>
+      </c>
+      <c r="C17" s="3">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="3">
+        <v>805</v>
+      </c>
+      <c r="C18" s="3">
+        <v>1</v>
+      </c>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="H18" s="1"/>
+      <c r="K18" s="1"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="3">
+        <v>805</v>
+      </c>
+      <c r="C19" s="3">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3">
+        <v>60</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="3">
+        <v>1</v>
+      </c>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="3">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="3">
+        <v>1</v>
+      </c>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="3" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3">
-        <v>805</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>1210</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="F6" s="7"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7">
-        <v>805</v>
-      </c>
-      <c r="C7">
-        <v>10</v>
-      </c>
-      <c r="D7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9">
-        <v>2</v>
-      </c>
-      <c r="D9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10">
-        <v>2</v>
-      </c>
-      <c r="D10" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11">
-        <v>10</v>
-      </c>
-      <c r="D11" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12">
-        <v>10</v>
-      </c>
-      <c r="D12" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13">
-        <v>805</v>
-      </c>
-      <c r="C13">
-        <v>10</v>
-      </c>
-      <c r="D13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14">
-        <v>805</v>
-      </c>
-      <c r="C14">
-        <v>10</v>
-      </c>
-      <c r="D14" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15">
-        <v>805</v>
-      </c>
-      <c r="C15">
-        <v>10</v>
-      </c>
-      <c r="D15" t="s">
-        <v>33</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16">
-        <v>805</v>
-      </c>
-      <c r="C16">
-        <v>10</v>
-      </c>
-      <c r="D16" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17">
-        <v>805</v>
-      </c>
-      <c r="C17">
-        <v>10</v>
-      </c>
-      <c r="D17" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18">
-        <v>805</v>
-      </c>
-      <c r="C18">
-        <v>10</v>
-      </c>
-      <c r="D18" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19">
-        <v>805</v>
-      </c>
-      <c r="C19">
-        <v>10</v>
-      </c>
-      <c r="D19">
-        <v>60</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>41</v>
-      </c>
-      <c r="B20" t="s">
-        <v>42</v>
-      </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-      <c r="D20" t="s">
-        <v>43</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>44</v>
-      </c>
-      <c r="B21" t="s">
-        <v>45</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-      <c r="D21" t="s">
-        <v>46</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" t="s">
-        <v>48</v>
-      </c>
-      <c r="C22">
-        <v>1</v>
-      </c>
-      <c r="D22" t="s">
-        <v>49</v>
-      </c>
-      <c r="E22" t="s">
-        <v>60</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E8" r:id="rId1" display="https://www.mouser.com/Search/Refine?Keyword=621-DF01ST" xr:uid="{12D3BB83-1EFC-45BD-B14F-097F679F2BF1}"/>
+    <hyperlink ref="F8" r:id="rId1" display="https://www.mouser.com/Search/Refine?Keyword=621-DF01ST" xr:uid="{12D3BB83-1EFC-45BD-B14F-097F679F2BF1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>